<commit_message>
Daily Activity Tracker 7Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="369" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A7A5D7C-3359-428B-9DF6-CF076F7FBC83}"/>
+  <xr:revisionPtr revIDLastSave="383" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{294293E9-95E9-4C58-970D-8DAD3FA05D17}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="85">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>Studied for exams.</t>
+  </si>
+  <si>
+    <t>Gave two CA's.</t>
   </si>
 </sst>
 </file>
@@ -2266,27 +2269,51 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+    <row r="32" spans="1:14" ht="15">
+      <c r="A32" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B32" s="14">
+        <v>480</v>
+      </c>
+      <c r="C32" s="14">
+        <v>10</v>
+      </c>
+      <c r="D32" s="14">
+        <v>120</v>
+      </c>
+      <c r="E32" s="14">
+        <v>0</v>
+      </c>
+      <c r="F32" s="14">
+        <v>400</v>
+      </c>
+      <c r="G32" s="14">
+        <v>8</v>
+      </c>
+      <c r="H32" s="14">
+        <v>0</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
+        <v>430</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 8Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="383" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{294293E9-95E9-4C58-970D-8DAD3FA05D17}"/>
+  <xr:revisionPtr revIDLastSave="396" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF96C7DF-05A8-4624-847D-43FB47959E38}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>Gave two CA's.</t>
+  </si>
+  <si>
+    <t>Gave one CA.</t>
   </si>
 </sst>
 </file>
@@ -2315,27 +2318,51 @@
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+    <row r="33" spans="1:14" ht="15">
+      <c r="A33" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B33" s="14">
+        <v>520</v>
+      </c>
+      <c r="C33" s="14">
+        <v>20</v>
+      </c>
+      <c r="D33" s="14">
+        <v>120</v>
+      </c>
+      <c r="E33" s="14">
+        <v>60</v>
+      </c>
+      <c r="F33" s="14">
+        <v>300</v>
+      </c>
+      <c r="G33" s="14">
+        <v>6</v>
+      </c>
+      <c r="H33" s="14">
+        <v>30</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 9Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="396" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF96C7DF-05A8-4624-847D-43FB47959E38}"/>
+  <xr:revisionPtr revIDLastSave="410" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9648AF5-C0ED-4CE2-ACB2-FA8ABF9A6BB5}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2364,27 +2364,51 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+    <row r="34" spans="1:14" ht="15">
+      <c r="A34" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B34" s="14">
+        <v>540</v>
+      </c>
+      <c r="C34" s="14">
+        <v>20</v>
+      </c>
+      <c r="D34" s="14">
+        <v>60</v>
+      </c>
+      <c r="E34" s="14">
+        <v>120</v>
+      </c>
+      <c r="F34" s="14">
+        <v>250</v>
+      </c>
+      <c r="G34" s="14">
+        <v>5</v>
+      </c>
+      <c r="H34" s="14">
+        <v>30</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="13"/>

</xml_diff>

<commit_message>
Dai;y Activity Tracker 10Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="410" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9648AF5-C0ED-4CE2-ACB2-FA8ABF9A6BB5}"/>
+  <xr:revisionPtr revIDLastSave="423" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7C449A0-90A2-44D8-AE20-EE5313E04419}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>Gave one CA.</t>
+  </si>
+  <si>
+    <t>Attended Freshers party.</t>
   </si>
 </sst>
 </file>
@@ -2410,27 +2413,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+    <row r="35" spans="1:14" ht="15">
+      <c r="A35" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B35" s="14">
+        <v>550</v>
+      </c>
+      <c r="C35" s="14">
+        <v>30</v>
+      </c>
+      <c r="D35" s="14">
+        <v>60</v>
+      </c>
+      <c r="E35" s="14">
+        <v>60</v>
+      </c>
+      <c r="F35" s="14">
+        <v>100</v>
+      </c>
+      <c r="G35" s="14">
+        <v>2</v>
+      </c>
+      <c r="H35" s="14">
+        <v>60</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
+        <v>580</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 11Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="423" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7C449A0-90A2-44D8-AE20-EE5313E04419}"/>
+  <xr:revisionPtr revIDLastSave="435" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1093D3BA-6E56-49AD-833D-0850920C7290}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2459,27 +2459,51 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+    <row r="36" spans="1:14" ht="15">
+      <c r="A36" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B36" s="14">
+        <v>500</v>
+      </c>
+      <c r="C36" s="14">
+        <v>30</v>
+      </c>
+      <c r="D36" s="14">
+        <v>120</v>
+      </c>
+      <c r="E36" s="14">
+        <v>120</v>
+      </c>
+      <c r="F36" s="14">
+        <v>150</v>
+      </c>
+      <c r="G36" s="14">
+        <v>3</v>
+      </c>
+      <c r="H36" s="14">
+        <v>30</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
+        <v>490</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 12Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="435" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1093D3BA-6E56-49AD-833D-0850920C7290}"/>
+  <xr:revisionPtr revIDLastSave="447" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06712DCD-6F6D-43D8-83B0-31F8DE4CE7B2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Attended Freshers party.</t>
+  </si>
+  <si>
+    <t>Learning new skills.</t>
   </si>
 </sst>
 </file>
@@ -2505,27 +2508,51 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+    <row r="37" spans="1:14" ht="15">
+      <c r="A37" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B37" s="14">
+        <v>620</v>
+      </c>
+      <c r="C37" s="14">
+        <v>30</v>
+      </c>
+      <c r="D37" s="14">
+        <v>180</v>
+      </c>
+      <c r="E37" s="14">
+        <v>120</v>
+      </c>
+      <c r="F37" s="14">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14">
+        <v>0</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
+        <v>490</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 13Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="447" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06712DCD-6F6D-43D8-83B0-31F8DE4CE7B2}"/>
+  <xr:revisionPtr revIDLastSave="459" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7609F135-996E-42B3-9873-3364B4AA85E7}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>Learning new skills.</t>
+  </si>
+  <si>
+    <t>Went for shopping.</t>
   </si>
 </sst>
 </file>
@@ -2554,27 +2557,51 @@
         <v>87</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+    <row r="38" spans="1:14" ht="15">
+      <c r="A38" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B38" s="14">
+        <v>650</v>
+      </c>
+      <c r="C38" s="14">
+        <v>30</v>
+      </c>
+      <c r="D38" s="14">
+        <v>120</v>
+      </c>
+      <c r="E38" s="14">
+        <v>120</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>30</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
+        <v>490</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 14Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="459" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7609F135-996E-42B3-9873-3364B4AA85E7}"/>
+  <xr:revisionPtr revIDLastSave="473" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D11EE37-EA73-4B1D-A378-EECC7D6097C9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2603,27 +2603,51 @@
         <v>88</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+    <row r="39" spans="1:14" ht="15">
+      <c r="A39" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B39" s="14">
+        <v>520</v>
+      </c>
+      <c r="C39" s="14">
+        <v>20</v>
+      </c>
+      <c r="D39" s="14">
+        <v>120</v>
+      </c>
+      <c r="E39" s="14">
+        <v>60</v>
+      </c>
+      <c r="F39" s="14">
+        <v>400</v>
+      </c>
+      <c r="G39" s="14">
+        <v>8</v>
+      </c>
+      <c r="H39" s="14">
+        <v>0</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
+        <v>320</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 15Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30509"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="473" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D11EE37-EA73-4B1D-A378-EECC7D6097C9}"/>
+  <xr:revisionPtr revIDLastSave="487" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9E3B09E-2EAC-49CD-9A68-5A67A6158ED9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -307,6 +307,9 @@
   </si>
   <si>
     <t>Went for shopping.</t>
+  </si>
+  <si>
+    <t>Gave one CA exam.</t>
   </si>
 </sst>
 </file>
@@ -2649,27 +2652,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+    <row r="40" spans="1:14" ht="15">
+      <c r="A40" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B40" s="14">
+        <v>520</v>
+      </c>
+      <c r="C40" s="14">
+        <v>30</v>
+      </c>
+      <c r="D40" s="14">
+        <v>120</v>
+      </c>
+      <c r="E40" s="14">
+        <v>60</v>
+      </c>
+      <c r="F40" s="14">
+        <v>300</v>
+      </c>
+      <c r="G40" s="14">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14">
+        <v>0</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 18Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="487" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9E3B09E-2EAC-49CD-9A68-5A67A6158ED9}"/>
+  <xr:revisionPtr revIDLastSave="499" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{438DF9B7-E1E0-423F-98FB-8D0883E77D61}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>Gave one CA exam.</t>
+  </si>
+  <si>
+    <t>Attended all classes.</t>
   </si>
 </sst>
 </file>
@@ -2698,27 +2701,51 @@
         <v>89</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+    <row r="41" spans="1:14" ht="15">
+      <c r="A41" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B41" s="14">
+        <v>540</v>
+      </c>
+      <c r="C41" s="14">
+        <v>30</v>
+      </c>
+      <c r="D41" s="14">
+        <v>120</v>
+      </c>
+      <c r="E41" s="14">
+        <v>30</v>
+      </c>
+      <c r="F41" s="14">
+        <v>300</v>
+      </c>
+      <c r="G41" s="14">
+        <v>6</v>
+      </c>
+      <c r="H41" s="14">
+        <v>20</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
+        <v>400</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 17Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="499" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{438DF9B7-E1E0-423F-98FB-8D0883E77D61}"/>
+  <xr:revisionPtr revIDLastSave="511" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7819B3B-DA7B-409E-8556-064981C167C0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="92">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -313,6 +313,9 @@
   </si>
   <si>
     <t>Attended all classes.</t>
+  </si>
+  <si>
+    <t>Studied for my analytical exam.</t>
   </si>
 </sst>
 </file>
@@ -2747,27 +2750,51 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+    <row r="42" spans="1:14" ht="15">
+      <c r="A42" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B42" s="14">
+        <v>520</v>
+      </c>
+      <c r="C42" s="14">
+        <v>40</v>
+      </c>
+      <c r="D42" s="14">
+        <v>240</v>
+      </c>
+      <c r="E42" s="14">
+        <v>30</v>
+      </c>
+      <c r="F42" s="14">
+        <v>150</v>
+      </c>
+      <c r="G42" s="14">
+        <v>3</v>
+      </c>
+      <c r="H42" s="14">
+        <v>30</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
+        <v>430</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="13"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 19Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="93">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3464,26 +3464,50 @@
       </c>
     </row>
     <row r="44" ht="17" spans="1:14">
-      <c r="A44" s="8"/>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="9"/>
-      <c r="I44" s="12" t="str">
+      <c r="A44" s="8">
+        <v>46284</v>
+      </c>
+      <c r="B44" s="9">
+        <v>480</v>
+      </c>
+      <c r="C44" s="9">
+        <v>20</v>
+      </c>
+      <c r="D44" s="9">
+        <v>150</v>
+      </c>
+      <c r="E44" s="9">
+        <v>120</v>
+      </c>
+      <c r="F44" s="9">
+        <v>0</v>
+      </c>
+      <c r="G44" s="9">
+        <v>0</v>
+      </c>
+      <c r="H44" s="9">
+        <v>30</v>
+      </c>
+      <c r="I44" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="12" t="str">
+        <v>800</v>
+      </c>
+      <c r="J44" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="13"/>
-      <c r="L44" s="13"/>
-      <c r="M44" s="13"/>
-      <c r="N44" s="15"/>
+        <v>640</v>
+      </c>
+      <c r="K44" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L44" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M44" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N44" s="15" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="45" ht="17" spans="1:14">
       <c r="A45" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 21Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -307,6 +307,9 @@
   </si>
   <si>
     <t>Going through cold and feever</t>
+  </si>
+  <si>
+    <t>Attended all class and tired after evening classes.</t>
   </si>
 </sst>
 </file>
@@ -3510,48 +3513,96 @@
       </c>
     </row>
     <row r="45" ht="17" spans="1:14">
-      <c r="A45" s="8"/>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="12" t="str">
+      <c r="A45" s="8">
+        <v>46285</v>
+      </c>
+      <c r="B45" s="9">
+        <v>550</v>
+      </c>
+      <c r="C45" s="9">
+        <v>30</v>
+      </c>
+      <c r="D45" s="9">
+        <v>180</v>
+      </c>
+      <c r="E45" s="9">
+        <v>160</v>
+      </c>
+      <c r="F45" s="9">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9">
+        <v>40</v>
+      </c>
+      <c r="I45" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="12" t="str">
+        <v>960</v>
+      </c>
+      <c r="J45" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="13"/>
-      <c r="L45" s="13"/>
-      <c r="M45" s="13"/>
-      <c r="N45" s="15"/>
-    </row>
-    <row r="46" ht="17" spans="1:14">
-      <c r="A46" s="8"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9"/>
-      <c r="I46" s="12" t="str">
+        <v>480</v>
+      </c>
+      <c r="K45" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L45" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M45" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N45" s="15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46" ht="34" spans="1:14">
+      <c r="A46" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B46" s="9">
+        <v>450</v>
+      </c>
+      <c r="C46" s="9">
+        <v>30</v>
+      </c>
+      <c r="D46" s="9">
+        <v>120</v>
+      </c>
+      <c r="E46" s="9">
+        <v>90</v>
+      </c>
+      <c r="F46" s="9">
+        <v>400</v>
+      </c>
+      <c r="G46" s="9">
+        <v>8</v>
+      </c>
+      <c r="H46" s="9">
+        <v>20</v>
+      </c>
+      <c r="I46" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="12" t="str">
+        <v>1110</v>
+      </c>
+      <c r="J46" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="13"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="13"/>
-      <c r="N46" s="15"/>
+        <v>330</v>
+      </c>
+      <c r="K46" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="L46" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="M46" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N46" s="15" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="47" ht="17" spans="1:14">
       <c r="A47" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 22Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>Attended all class and tired after evening classes.</t>
+  </si>
+  <si>
+    <t>Good day. Attended all classes</t>
   </si>
 </sst>
 </file>
@@ -3605,26 +3608,50 @@
       </c>
     </row>
     <row r="47" ht="17" spans="1:14">
-      <c r="A47" s="8"/>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="9"/>
-      <c r="I47" s="12" t="str">
+      <c r="A47" s="8">
+        <v>46287</v>
+      </c>
+      <c r="B47" s="9">
+        <v>520</v>
+      </c>
+      <c r="C47" s="9">
+        <v>30</v>
+      </c>
+      <c r="D47" s="9">
+        <v>180</v>
+      </c>
+      <c r="E47" s="9">
+        <v>90</v>
+      </c>
+      <c r="F47" s="9">
+        <v>300</v>
+      </c>
+      <c r="G47" s="9">
+        <v>6</v>
+      </c>
+      <c r="H47" s="9">
+        <v>40</v>
+      </c>
+      <c r="I47" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="12" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J47" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="13"/>
-      <c r="L47" s="13"/>
-      <c r="M47" s="13"/>
-      <c r="N47" s="15"/>
+        <v>280</v>
+      </c>
+      <c r="K47" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L47" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M47" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N47" s="15" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="48" ht="17" spans="1:14">
       <c r="A48" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 23Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="96">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -313,6 +313,9 @@
   </si>
   <si>
     <t>Good day. Attended all classes</t>
+  </si>
+  <si>
+    <t>Worked on my python project.</t>
   </si>
 </sst>
 </file>
@@ -3654,26 +3657,50 @@
       </c>
     </row>
     <row r="48" ht="17" spans="1:14">
-      <c r="A48" s="8"/>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="9"/>
-      <c r="I48" s="12" t="str">
+      <c r="A48" s="8">
+        <v>46288</v>
+      </c>
+      <c r="B48" s="9">
+        <v>560</v>
+      </c>
+      <c r="C48" s="9">
+        <v>20</v>
+      </c>
+      <c r="D48" s="9">
+        <v>120</v>
+      </c>
+      <c r="E48" s="9">
+        <v>60</v>
+      </c>
+      <c r="F48" s="9">
+        <v>300</v>
+      </c>
+      <c r="G48" s="9">
+        <v>6</v>
+      </c>
+      <c r="H48" s="9">
+        <v>30</v>
+      </c>
+      <c r="I48" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="12" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J48" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="13"/>
-      <c r="L48" s="13"/>
-      <c r="M48" s="13"/>
-      <c r="N48" s="15"/>
+        <v>350</v>
+      </c>
+      <c r="K48" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L48" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M48" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N48" s="15" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="49" ht="17" spans="1:14">
       <c r="A49" s="8"/>

</xml_diff>

<commit_message>
Daly Activity Tracker 24Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="96">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -135,7 +135,7 @@
     <t>Course / Section:</t>
   </si>
   <si>
-    <t>MCA / SD1P2631</t>
+    <t>MCA / D1P2631</t>
   </si>
   <si>
     <t>Month:</t>
@@ -315,7 +315,7 @@
     <t>Good day. Attended all classes</t>
   </si>
   <si>
-    <t>Worked on my python project.</t>
+    <t>Prepared for my CA exams</t>
   </si>
 </sst>
 </file>
@@ -3703,25 +3703,47 @@
       </c>
     </row>
     <row r="49" ht="17" spans="1:14">
-      <c r="A49" s="8"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
-      <c r="H49" s="9"/>
-      <c r="I49" s="12" t="str">
+      <c r="A49" s="8">
+        <v>46289</v>
+      </c>
+      <c r="B49" s="9">
+        <v>520</v>
+      </c>
+      <c r="C49" s="9">
+        <v>30</v>
+      </c>
+      <c r="D49" s="9">
+        <v>180</v>
+      </c>
+      <c r="E49" s="9">
+        <v>60</v>
+      </c>
+      <c r="F49" s="9">
+        <v>150</v>
+      </c>
+      <c r="G49" s="9">
+        <v>3</v>
+      </c>
+      <c r="H49" s="9">
+        <v>30</v>
+      </c>
+      <c r="I49" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="12" t="str">
+        <v>970</v>
+      </c>
+      <c r="J49" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="13"/>
-      <c r="L49" s="13"/>
-      <c r="M49" s="13"/>
+        <v>470</v>
+      </c>
+      <c r="K49" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L49" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M49" s="13" t="s">
+        <v>59</v>
+      </c>
       <c r="N49" s="15"/>
     </row>
     <row r="50" ht="17" spans="1:14">

</xml_diff>

<commit_message>
Daily Activity Tracker 25Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -316,6 +316,9 @@
   </si>
   <si>
     <t>Prepared for my CA exams</t>
+  </si>
+  <si>
+    <t>Had good rest after all classes.</t>
   </si>
 </sst>
 </file>
@@ -3744,29 +3747,55 @@
       <c r="M49" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="N49" s="15"/>
+      <c r="N49" s="15" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="50" ht="17" spans="1:14">
-      <c r="A50" s="8"/>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="9"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="12" t="str">
+      <c r="A50" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B50" s="9">
+        <v>520</v>
+      </c>
+      <c r="C50" s="9">
+        <v>30</v>
+      </c>
+      <c r="D50" s="9">
+        <v>180</v>
+      </c>
+      <c r="E50" s="9">
+        <v>30</v>
+      </c>
+      <c r="F50" s="9">
+        <v>200</v>
+      </c>
+      <c r="G50" s="9">
+        <v>4</v>
+      </c>
+      <c r="H50" s="9">
+        <v>30</v>
+      </c>
+      <c r="I50" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="12" t="str">
+        <v>990</v>
+      </c>
+      <c r="J50" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="13"/>
-      <c r="L50" s="13"/>
-      <c r="M50" s="13"/>
-      <c r="N50" s="15"/>
+        <v>450</v>
+      </c>
+      <c r="K50" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L50" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M50" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N50" s="15" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="51" ht="17" spans="1:14">
       <c r="A51" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 28Sept
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AEEF270-F1E9-B040-9745-E19DDB301BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1000001_{E2FAA0BC-1B5C-664B-8106-7EA3B6E1C992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28260" windowHeight="13420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -321,13 +321,16 @@
   <si>
     <t>Had good rest after all classes.</t>
   </si>
+  <si>
+    <t>Going home.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -463,13 +466,13 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -498,9 +501,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -985,74 +988,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <v>12607891</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
       <c r="E3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" ht="39.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -3215,26 +3218,50 @@
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A52" s="5"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="9" t="str">
+      <c r="A52" s="5">
+        <v>46293</v>
+      </c>
+      <c r="B52" s="6">
+        <v>450</v>
+      </c>
+      <c r="C52" s="6">
+        <v>20</v>
+      </c>
+      <c r="D52" s="6">
+        <v>0</v>
+      </c>
+      <c r="E52" s="6">
+        <v>0</v>
+      </c>
+      <c r="F52" s="6">
+        <v>0</v>
+      </c>
+      <c r="G52" s="6">
+        <v>0</v>
+      </c>
+      <c r="H52" s="6">
+        <v>60</v>
+      </c>
+      <c r="I52" s="9">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="9" t="str">
+        <v>530</v>
+      </c>
+      <c r="J52" s="9">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="10"/>
-      <c r="N52" s="12"/>
+        <v>910</v>
+      </c>
+      <c r="K52" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="L52" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="M52" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="N52" s="12" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="5"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 2Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t>Reached home and tired</t>
+  </si>
+  <si>
+    <t>Preparing for MTE</t>
   </si>
 </sst>
 </file>
@@ -3942,26 +3945,50 @@
       </c>
     </row>
     <row r="54" ht="17" spans="1:14">
-      <c r="A54" s="8"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="9"/>
-      <c r="H54" s="9"/>
-      <c r="I54" s="12" t="str">
+      <c r="A54" s="8">
+        <v>46297</v>
+      </c>
+      <c r="B54" s="9">
+        <v>570</v>
+      </c>
+      <c r="C54" s="9">
+        <v>30</v>
+      </c>
+      <c r="D54" s="9">
+        <v>180</v>
+      </c>
+      <c r="E54" s="9">
+        <v>60</v>
+      </c>
+      <c r="F54" s="9">
+        <v>0</v>
+      </c>
+      <c r="G54" s="9">
+        <v>0</v>
+      </c>
+      <c r="H54" s="9">
+        <v>60</v>
+      </c>
+      <c r="I54" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="12" t="str">
+        <v>900</v>
+      </c>
+      <c r="J54" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="13"/>
-      <c r="L54" s="13"/>
-      <c r="M54" s="13"/>
-      <c r="N54" s="15"/>
+        <v>540</v>
+      </c>
+      <c r="K54" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L54" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M54" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N54" s="15" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="55" ht="17" spans="1:14">
       <c r="A55" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 03Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3991,26 +3991,50 @@
       </c>
     </row>
     <row r="55" ht="17" spans="1:14">
-      <c r="A55" s="8"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
-      <c r="G55" s="9"/>
-      <c r="H55" s="9"/>
-      <c r="I55" s="12" t="str">
+      <c r="A55" s="8">
+        <v>46298</v>
+      </c>
+      <c r="B55" s="9">
+        <v>540</v>
+      </c>
+      <c r="C55" s="9">
+        <v>30</v>
+      </c>
+      <c r="D55" s="9">
+        <v>180</v>
+      </c>
+      <c r="E55" s="9">
+        <v>120</v>
+      </c>
+      <c r="F55" s="9">
+        <v>0</v>
+      </c>
+      <c r="G55" s="9">
+        <v>0</v>
+      </c>
+      <c r="H55" s="9">
+        <v>60</v>
+      </c>
+      <c r="I55" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="12" t="str">
+        <v>930</v>
+      </c>
+      <c r="J55" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="13"/>
-      <c r="L55" s="13"/>
-      <c r="M55" s="13"/>
-      <c r="N55" s="15"/>
+        <v>510</v>
+      </c>
+      <c r="K55" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L55" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M55" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N55" s="15" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="56" ht="17" spans="1:14">
       <c r="A56" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 04Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4037,26 +4037,50 @@
       </c>
     </row>
     <row r="56" ht="17" spans="1:14">
-      <c r="A56" s="8"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="12" t="str">
+      <c r="A56" s="8">
+        <v>46299</v>
+      </c>
+      <c r="B56" s="9">
+        <v>570</v>
+      </c>
+      <c r="C56" s="9">
+        <v>20</v>
+      </c>
+      <c r="D56" s="9">
+        <v>150</v>
+      </c>
+      <c r="E56" s="9">
+        <v>60</v>
+      </c>
+      <c r="F56" s="9">
+        <v>0</v>
+      </c>
+      <c r="G56" s="9">
+        <v>0</v>
+      </c>
+      <c r="H56" s="9">
+        <v>30</v>
+      </c>
+      <c r="I56" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="12" t="str">
+        <v>830</v>
+      </c>
+      <c r="J56" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="13"/>
-      <c r="L56" s="13"/>
-      <c r="M56" s="13"/>
-      <c r="N56" s="15"/>
+        <v>610</v>
+      </c>
+      <c r="K56" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L56" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M56" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N56" s="15" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="57" ht="17" spans="1:14">
       <c r="A57" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 05Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="17880" windowHeight="13420" tabRatio="500" firstSheet="1" activeTab="1"/>
+    <workbookView windowWidth="28260" windowHeight="13420" tabRatio="500" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4083,26 +4083,50 @@
       </c>
     </row>
     <row r="57" ht="17" spans="1:14">
-      <c r="A57" s="8"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="12" t="str">
+      <c r="A57" s="8">
+        <v>46300</v>
+      </c>
+      <c r="B57" s="9">
+        <v>520</v>
+      </c>
+      <c r="C57" s="9">
+        <v>30</v>
+      </c>
+      <c r="D57" s="9">
+        <v>120</v>
+      </c>
+      <c r="E57" s="9">
+        <v>60</v>
+      </c>
+      <c r="F57" s="9">
+        <v>400</v>
+      </c>
+      <c r="G57" s="9">
+        <v>8</v>
+      </c>
+      <c r="H57" s="9">
+        <v>30</v>
+      </c>
+      <c r="I57" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="12" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J57" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="13"/>
-      <c r="L57" s="13"/>
-      <c r="M57" s="13"/>
-      <c r="N57" s="15"/>
+        <v>280</v>
+      </c>
+      <c r="K57" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L57" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M57" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N57" s="15" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="58" ht="17" spans="1:14">
       <c r="A58" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 06Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="100">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4129,26 +4129,50 @@
       </c>
     </row>
     <row r="58" ht="17" spans="1:14">
-      <c r="A58" s="8"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="12" t="str">
+      <c r="A58" s="8">
+        <v>46301</v>
+      </c>
+      <c r="B58" s="9">
+        <v>480</v>
+      </c>
+      <c r="C58" s="9">
+        <v>30</v>
+      </c>
+      <c r="D58" s="9">
+        <v>60</v>
+      </c>
+      <c r="E58" s="9">
+        <v>60</v>
+      </c>
+      <c r="F58" s="9">
+        <v>300</v>
+      </c>
+      <c r="G58" s="9">
+        <v>6</v>
+      </c>
+      <c r="H58" s="9">
+        <v>39</v>
+      </c>
+      <c r="I58" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="12" t="str">
+        <v>969</v>
+      </c>
+      <c r="J58" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="13"/>
-      <c r="L58" s="13"/>
-      <c r="M58" s="13"/>
-      <c r="N58" s="15"/>
+        <v>471</v>
+      </c>
+      <c r="K58" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L58" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M58" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N58" s="15" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="59" ht="17" spans="1:14">
       <c r="A59" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 07Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="101">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>Preparing for MTE</t>
+  </si>
+  <si>
+    <t>Good day. Attended all classes.</t>
   </si>
 </sst>
 </file>
@@ -4175,26 +4178,50 @@
       </c>
     </row>
     <row r="59" ht="17" spans="1:14">
-      <c r="A59" s="8"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="12" t="str">
+      <c r="A59" s="8">
+        <v>46302</v>
+      </c>
+      <c r="B59" s="9">
+        <v>520</v>
+      </c>
+      <c r="C59" s="9">
+        <v>30</v>
+      </c>
+      <c r="D59" s="9">
+        <v>120</v>
+      </c>
+      <c r="E59" s="9">
+        <v>60</v>
+      </c>
+      <c r="F59" s="9">
+        <v>300</v>
+      </c>
+      <c r="G59" s="9">
+        <v>6</v>
+      </c>
+      <c r="H59" s="9">
+        <v>40</v>
+      </c>
+      <c r="I59" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="12" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J59" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="13"/>
-      <c r="L59" s="13"/>
-      <c r="M59" s="13"/>
-      <c r="N59" s="15"/>
+        <v>370</v>
+      </c>
+      <c r="K59" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L59" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M59" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N59" s="15" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="60" ht="17" spans="1:14">
       <c r="A60" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 08Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="102">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -331,6 +331,9 @@
   </si>
   <si>
     <t>Good day. Attended all classes.</t>
+  </si>
+  <si>
+    <t>Studied and watched movie.</t>
   </si>
 </sst>
 </file>
@@ -4224,26 +4227,50 @@
       </c>
     </row>
     <row r="60" ht="17" spans="1:14">
-      <c r="A60" s="8"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="12" t="str">
+      <c r="A60" s="8">
+        <v>46303</v>
+      </c>
+      <c r="B60" s="9">
+        <v>520</v>
+      </c>
+      <c r="C60" s="9">
+        <v>20</v>
+      </c>
+      <c r="D60" s="9">
+        <v>120</v>
+      </c>
+      <c r="E60" s="9">
+        <v>120</v>
+      </c>
+      <c r="F60" s="9">
+        <v>0</v>
+      </c>
+      <c r="G60" s="9">
+        <v>0</v>
+      </c>
+      <c r="H60" s="9">
+        <v>120</v>
+      </c>
+      <c r="I60" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="12" t="str">
+        <v>900</v>
+      </c>
+      <c r="J60" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K60" s="13"/>
-      <c r="L60" s="13"/>
-      <c r="M60" s="13"/>
-      <c r="N60" s="15"/>
+        <v>540</v>
+      </c>
+      <c r="K60" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L60" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M60" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N60" s="15" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="61" ht="17" spans="1:14">
       <c r="A61" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 09Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="102">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4273,26 +4273,50 @@
       </c>
     </row>
     <row r="61" ht="17" spans="1:14">
-      <c r="A61" s="8"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
-      <c r="H61" s="9"/>
-      <c r="I61" s="12" t="str">
+      <c r="A61" s="8">
+        <v>46304</v>
+      </c>
+      <c r="B61" s="9">
+        <v>480</v>
+      </c>
+      <c r="C61" s="9">
+        <v>30</v>
+      </c>
+      <c r="D61" s="9">
+        <v>150</v>
+      </c>
+      <c r="E61" s="9">
+        <v>0</v>
+      </c>
+      <c r="F61" s="9">
+        <v>0</v>
+      </c>
+      <c r="G61" s="9">
+        <v>0</v>
+      </c>
+      <c r="H61" s="9">
+        <v>60</v>
+      </c>
+      <c r="I61" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="12" t="str">
+        <v>720</v>
+      </c>
+      <c r="J61" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K61" s="13"/>
-      <c r="L61" s="13"/>
-      <c r="M61" s="13"/>
-      <c r="N61" s="15"/>
+        <v>720</v>
+      </c>
+      <c r="K61" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L61" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M61" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N61" s="15" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="62" ht="17" spans="1:14">
       <c r="A62" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 13Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>Studied and watched movie.</t>
+  </si>
+  <si>
+    <t>Prepared for my MTE.</t>
   </si>
 </sst>
 </file>
@@ -4319,26 +4322,50 @@
       </c>
     </row>
     <row r="62" ht="17" spans="1:14">
-      <c r="A62" s="8"/>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="12" t="str">
+      <c r="A62" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B62" s="9">
+        <v>520</v>
+      </c>
+      <c r="C62" s="9">
+        <v>30</v>
+      </c>
+      <c r="D62" s="9">
+        <v>240</v>
+      </c>
+      <c r="E62" s="9">
+        <v>0</v>
+      </c>
+      <c r="F62" s="9">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9">
+        <v>0</v>
+      </c>
+      <c r="H62" s="9">
+        <v>30</v>
+      </c>
+      <c r="I62" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="12" t="str">
+        <v>820</v>
+      </c>
+      <c r="J62" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="13"/>
-      <c r="L62" s="13"/>
-      <c r="M62" s="13"/>
-      <c r="N62" s="15"/>
+        <v>620</v>
+      </c>
+      <c r="K62" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L62" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M62" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N62" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="63" ht="17" spans="1:14">
       <c r="A63" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 14Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4368,26 +4368,50 @@
       </c>
     </row>
     <row r="63" ht="17" spans="1:14">
-      <c r="A63" s="8"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="12" t="str">
+      <c r="A63" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B63" s="9">
+        <v>520</v>
+      </c>
+      <c r="C63" s="9">
+        <v>20</v>
+      </c>
+      <c r="D63" s="9">
+        <v>240</v>
+      </c>
+      <c r="E63" s="9">
+        <v>0</v>
+      </c>
+      <c r="F63" s="9">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9">
+        <v>0</v>
+      </c>
+      <c r="H63" s="9">
+        <v>40</v>
+      </c>
+      <c r="I63" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="12" t="str">
+        <v>820</v>
+      </c>
+      <c r="J63" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="13"/>
-      <c r="L63" s="13"/>
-      <c r="M63" s="13"/>
-      <c r="N63" s="15"/>
+        <v>620</v>
+      </c>
+      <c r="K63" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L63" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M63" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N63" s="15" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="64" ht="17" spans="1:14">
       <c r="A64" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 15Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="103">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4323,7 +4323,7 @@
     </row>
     <row r="62" ht="17" spans="1:14">
       <c r="A62" s="8">
-        <v>46278</v>
+        <v>46308</v>
       </c>
       <c r="B62" s="9">
         <v>520</v>
@@ -4369,7 +4369,7 @@
     </row>
     <row r="63" ht="17" spans="1:14">
       <c r="A63" s="8">
-        <v>46279</v>
+        <v>46309</v>
       </c>
       <c r="B63" s="9">
         <v>520</v>
@@ -4414,26 +4414,50 @@
       </c>
     </row>
     <row r="64" ht="17" spans="1:14">
-      <c r="A64" s="8"/>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="12" t="str">
+      <c r="A64" s="8">
+        <v>46310</v>
+      </c>
+      <c r="B64" s="9">
+        <v>480</v>
+      </c>
+      <c r="C64" s="9">
+        <v>30</v>
+      </c>
+      <c r="D64" s="9">
+        <v>200</v>
+      </c>
+      <c r="E64" s="9">
+        <v>0</v>
+      </c>
+      <c r="F64" s="9">
+        <v>0</v>
+      </c>
+      <c r="G64" s="9">
+        <v>0</v>
+      </c>
+      <c r="H64" s="9">
+        <v>0</v>
+      </c>
+      <c r="I64" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="12" t="str">
+        <v>710</v>
+      </c>
+      <c r="J64" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K64" s="13"/>
-      <c r="L64" s="13"/>
-      <c r="M64" s="13"/>
-      <c r="N64" s="15"/>
+        <v>730</v>
+      </c>
+      <c r="K64" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L64" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M64" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N64" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="65" ht="17" spans="1:14">
       <c r="A65" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 16Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="104">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>Prepared for my MTE.</t>
+  </si>
+  <si>
+    <t>Played cricket today.</t>
   </si>
 </sst>
 </file>
@@ -4460,26 +4463,50 @@
       </c>
     </row>
     <row r="65" ht="17" spans="1:14">
-      <c r="A65" s="8"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="12" t="str">
+      <c r="A65" s="8">
+        <v>46311</v>
+      </c>
+      <c r="B65" s="9">
+        <v>500</v>
+      </c>
+      <c r="C65" s="9">
+        <v>30</v>
+      </c>
+      <c r="D65" s="9">
+        <v>240</v>
+      </c>
+      <c r="E65" s="9">
+        <v>0</v>
+      </c>
+      <c r="F65" s="9">
+        <v>0</v>
+      </c>
+      <c r="G65" s="9">
+        <v>0</v>
+      </c>
+      <c r="H65" s="9">
+        <v>60</v>
+      </c>
+      <c r="I65" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="12" t="str">
+        <v>830</v>
+      </c>
+      <c r="J65" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K65" s="13"/>
-      <c r="L65" s="13"/>
-      <c r="M65" s="13"/>
-      <c r="N65" s="15"/>
+        <v>610</v>
+      </c>
+      <c r="K65" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L65" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M65" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N65" s="15" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="66" ht="17" spans="1:14">
       <c r="A66" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 19Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="104">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4509,26 +4509,50 @@
       </c>
     </row>
     <row r="66" ht="17" spans="1:14">
-      <c r="A66" s="8"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="12" t="str">
+      <c r="A66" s="8">
+        <v>46314</v>
+      </c>
+      <c r="B66" s="9">
+        <v>480</v>
+      </c>
+      <c r="C66" s="9">
+        <v>40</v>
+      </c>
+      <c r="D66" s="9">
+        <v>120</v>
+      </c>
+      <c r="E66" s="9">
+        <v>0</v>
+      </c>
+      <c r="F66" s="9">
+        <v>0</v>
+      </c>
+      <c r="G66" s="9">
+        <v>0</v>
+      </c>
+      <c r="H66" s="9">
+        <v>120</v>
+      </c>
+      <c r="I66" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="12" t="str">
+        <v>760</v>
+      </c>
+      <c r="J66" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K66" s="13"/>
-      <c r="L66" s="13"/>
-      <c r="M66" s="13"/>
-      <c r="N66" s="15"/>
+        <v>680</v>
+      </c>
+      <c r="K66" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L66" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M66" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N66" s="15" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="67" ht="17" spans="1:14">
       <c r="A67" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 20Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="105">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -340,6 +340,9 @@
   </si>
   <si>
     <t>Played cricket today.</t>
+  </si>
+  <si>
+    <t>Celebrating Dusshera.</t>
   </si>
 </sst>
 </file>
@@ -4555,26 +4558,50 @@
       </c>
     </row>
     <row r="67" ht="17" spans="1:14">
-      <c r="A67" s="8"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="12" t="str">
+      <c r="A67" s="8">
+        <v>46315</v>
+      </c>
+      <c r="B67" s="9">
+        <v>500</v>
+      </c>
+      <c r="C67" s="9">
+        <v>30</v>
+      </c>
+      <c r="D67" s="9">
+        <v>60</v>
+      </c>
+      <c r="E67" s="9">
+        <v>60</v>
+      </c>
+      <c r="F67" s="9">
+        <v>0</v>
+      </c>
+      <c r="G67" s="9">
+        <v>0</v>
+      </c>
+      <c r="H67" s="9">
+        <v>180</v>
+      </c>
+      <c r="I67" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="12" t="str">
+        <v>830</v>
+      </c>
+      <c r="J67" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K67" s="13"/>
-      <c r="L67" s="13"/>
-      <c r="M67" s="13"/>
-      <c r="N67" s="15"/>
+        <v>610</v>
+      </c>
+      <c r="K67" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="L67" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M67" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N67" s="15" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="68" ht="17" spans="1:14">
       <c r="A68" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 21Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="105">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4604,26 +4604,50 @@
       </c>
     </row>
     <row r="68" ht="17" spans="1:14">
-      <c r="A68" s="8"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="12" t="str">
+      <c r="A68" s="8">
+        <v>46316</v>
+      </c>
+      <c r="B68" s="9">
+        <v>480</v>
+      </c>
+      <c r="C68" s="9">
+        <v>30</v>
+      </c>
+      <c r="D68" s="9">
+        <v>120</v>
+      </c>
+      <c r="E68" s="9">
+        <v>120</v>
+      </c>
+      <c r="F68" s="9">
+        <v>0</v>
+      </c>
+      <c r="G68" s="9">
+        <v>0</v>
+      </c>
+      <c r="H68" s="9">
+        <v>60</v>
+      </c>
+      <c r="I68" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="12" t="str">
+        <v>810</v>
+      </c>
+      <c r="J68" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K68" s="13"/>
-      <c r="L68" s="13"/>
-      <c r="M68" s="13"/>
-      <c r="N68" s="15"/>
+        <v>630</v>
+      </c>
+      <c r="K68" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L68" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M68" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N68" s="15" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="69" ht="17" spans="1:14">
       <c r="A69" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 22Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="105">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4650,26 +4650,50 @@
       </c>
     </row>
     <row r="69" ht="17" spans="1:14">
-      <c r="A69" s="8"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="12" t="str">
+      <c r="A69" s="8">
+        <v>46317</v>
+      </c>
+      <c r="B69" s="9">
+        <v>560</v>
+      </c>
+      <c r="C69" s="9">
+        <v>20</v>
+      </c>
+      <c r="D69" s="9">
+        <v>180</v>
+      </c>
+      <c r="E69" s="9">
+        <v>60</v>
+      </c>
+      <c r="F69" s="9">
+        <v>0</v>
+      </c>
+      <c r="G69" s="9">
+        <v>0</v>
+      </c>
+      <c r="H69" s="9">
+        <v>60</v>
+      </c>
+      <c r="I69" s="12">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="12" t="str">
+        <v>880</v>
+      </c>
+      <c r="J69" s="12">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K69" s="13"/>
-      <c r="L69" s="13"/>
-      <c r="M69" s="13"/>
-      <c r="N69" s="15"/>
+        <v>560</v>
+      </c>
+      <c r="K69" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L69" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M69" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N69" s="15" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="70" ht="17" spans="1:14">
       <c r="A70" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 27Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="13400" tabRatio="500" firstSheet="1" activeTab="1"/>
+    <workbookView windowWidth="28260" windowHeight="13420" tabRatio="500" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="107">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t>Played football.</t>
+  </si>
+  <si>
+    <t>Tired after all classes.</t>
   </si>
 </sst>
 </file>
@@ -4791,26 +4794,50 @@
       </c>
     </row>
     <row r="72" ht="17" spans="1:14">
-      <c r="A72" s="8"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
-      <c r="H72" s="9"/>
-      <c r="I72" s="12" t="str">
+      <c r="A72" s="8">
+        <v>46322</v>
+      </c>
+      <c r="B72" s="9">
+        <v>540</v>
+      </c>
+      <c r="C72" s="9">
+        <v>30</v>
+      </c>
+      <c r="D72" s="9">
+        <v>180</v>
+      </c>
+      <c r="E72" s="9">
+        <v>60</v>
+      </c>
+      <c r="F72" s="9">
+        <v>300</v>
+      </c>
+      <c r="G72" s="9">
+        <v>6</v>
+      </c>
+      <c r="H72" s="9">
+        <v>50</v>
+      </c>
+      <c r="I72" s="12">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J72" s="12" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J72" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K72" s="13"/>
-      <c r="L72" s="13"/>
-      <c r="M72" s="13"/>
-      <c r="N72" s="15"/>
+        <v>280</v>
+      </c>
+      <c r="K72" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L72" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M72" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="N72" s="15" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="73" ht="17" spans="1:14">
       <c r="A73" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 28Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="107">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -4840,26 +4840,50 @@
       </c>
     </row>
     <row r="73" ht="17" spans="1:14">
-      <c r="A73" s="8"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="9"/>
-      <c r="H73" s="9"/>
-      <c r="I73" s="12" t="str">
+      <c r="A73" s="8">
+        <v>46323</v>
+      </c>
+      <c r="B73" s="9">
+        <v>480</v>
+      </c>
+      <c r="C73" s="9">
+        <v>20</v>
+      </c>
+      <c r="D73" s="9">
+        <v>180</v>
+      </c>
+      <c r="E73" s="9">
+        <v>60</v>
+      </c>
+      <c r="F73" s="9">
+        <v>250</v>
+      </c>
+      <c r="G73" s="9">
+        <v>5</v>
+      </c>
+      <c r="H73" s="9">
+        <v>30</v>
+      </c>
+      <c r="I73" s="12">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J73" s="12" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J73" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K73" s="13"/>
-      <c r="L73" s="13"/>
-      <c r="M73" s="13"/>
-      <c r="N73" s="15"/>
+        <v>420</v>
+      </c>
+      <c r="K73" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L73" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M73" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="N73" s="15" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="74" ht="17" spans="1:14">
       <c r="A74" s="8"/>

</xml_diff>

<commit_message>
Daily Activity Tracker 29Oct
</commit_message>
<xml_diff>
--- a/12607891.xlsx
+++ b/12607891.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="109">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -349,6 +349,12 @@
   </si>
   <si>
     <t>Tired after all classes.</t>
+  </si>
+  <si>
+    <t>Preparing for my MTE..</t>
+  </si>
+  <si>
+    <t>q</t>
   </si>
 </sst>
 </file>
@@ -4886,26 +4892,50 @@
       </c>
     </row>
     <row r="74" ht="17" spans="1:14">
-      <c r="A74" s="8"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="9"/>
-      <c r="F74" s="9"/>
-      <c r="G74" s="9"/>
-      <c r="H74" s="9"/>
-      <c r="I74" s="12" t="str">
+      <c r="A74" s="8">
+        <v>46324</v>
+      </c>
+      <c r="B74" s="9">
+        <v>450</v>
+      </c>
+      <c r="C74" s="9">
+        <v>30</v>
+      </c>
+      <c r="D74" s="9">
+        <v>240</v>
+      </c>
+      <c r="E74" s="9">
+        <v>0</v>
+      </c>
+      <c r="F74" s="9">
+        <v>150</v>
+      </c>
+      <c r="G74" s="9">
+        <v>3</v>
+      </c>
+      <c r="H74" s="9">
+        <v>40</v>
+      </c>
+      <c r="I74" s="12">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J74" s="12" t="str">
+        <v>910</v>
+      </c>
+      <c r="J74" s="12">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K74" s="13"/>
-      <c r="L74" s="13"/>
-      <c r="M74" s="13"/>
-      <c r="N74" s="15"/>
+        <v>530</v>
+      </c>
+      <c r="K74" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L74" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="M74" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="N74" s="15" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="75" ht="17" spans="1:14">
       <c r="A75" s="8"/>
@@ -4969,7 +4999,9 @@
         <v/>
       </c>
       <c r="K77" s="13"/>
-      <c r="L77" s="13"/>
+      <c r="L77" s="13" t="s">
+        <v>108</v>
+      </c>
       <c r="M77" s="13"/>
       <c r="N77" s="15"/>
     </row>

</xml_diff>